<commit_message>
Add wave presentation and update game content
</commit_message>
<xml_diff>
--- a/content/wave.xlsx
+++ b/content/wave.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
       <sz val="10"/>
     </font>
     <font>
@@ -119,10 +123,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -137,6 +141,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1344,9 +1349,9 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1377,27 +1382,23 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="A2" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>ENEMY_SKELETON_GOLD</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>MONSTERTYPE_BOSS</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>7판을 손으로 잡는다</t>
         </is>

</xml_diff>